<commit_message>
add tech files uplaod and info list
</commit_message>
<xml_diff>
--- a/back-end/mkd_works_service/komf_houses.xlsx
+++ b/back-end/mkd_works_service/komf_houses.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Housing Company Services(HCS)\back-end\mkd_works_service\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38D5175F-F37A-4C97-8CA6-D54141B01016}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7611AE05-6020-4E14-B0C5-BEF5C06DE334}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="22">
   <si>
     <t>Улица</t>
   </si>
@@ -88,6 +88,9 @@
   </si>
   <si>
     <t>20А</t>
+  </si>
+  <si>
+    <t>Площадь</t>
   </si>
 </sst>
 </file>
@@ -169,7 +172,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -177,6 +180,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -457,7 +461,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D60"/>
+  <dimension ref="A1:E60"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34.28515625" customWidth="1"/>
@@ -466,7 +470,7 @@
     <col min="4" max="4" width="18.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -479,8 +483,11 @@
       <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -488,7 +495,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -496,7 +503,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -504,7 +511,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -512,7 +519,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -520,7 +527,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -528,7 +535,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -536,7 +543,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -544,7 +551,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>7</v>
       </c>
@@ -552,7 +559,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>7</v>
       </c>
@@ -560,7 +567,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>7</v>
       </c>
@@ -568,7 +575,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>7</v>
       </c>
@@ -576,7 +583,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>7</v>
       </c>
@@ -584,7 +591,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>7</v>
       </c>
@@ -592,7 +599,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>7</v>
       </c>

</xml_diff>